<commit_message>
Update annotations for L4 -> LD "laminar dissecans"
</commit_message>
<xml_diff>
--- a/processed-data/05_spe_correct_cluster/10_spatial_registration_DLPFC/ERC_SpD_spatial_registration_Annotations.xlsx
+++ b/processed-data/05_spe_correct_cluster/10_spatial_registration_DLPFC/ERC_SpD_spatial_registration_Annotations.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10309"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://lieberinstitute-my.sharepoint.com/personal/louise_huuki_libd_org/Documents/LIBD_code/LFF_spatial_ERC/processed-data/05_spe_correct_cluster/10_spatial_registration_DLPFC/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="30" documentId="8_{A6B8FFDE-9993-5E49-A3D7-A78A78ED7963}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8C483E71-835C-314E-BB97-1F287326AEB0}"/>
+  <xr:revisionPtr revIDLastSave="31" documentId="8_{A6B8FFDE-9993-5E49-A3D7-A78A78ED7963}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{66F9A689-F83F-164C-8E66-69B4D30EDD03}"/>
   <bookViews>
     <workbookView xWindow="1100" yWindow="820" windowWidth="28040" windowHeight="17440" xr2:uid="{145CA205-9E01-CF4B-AF13-75949B1F1E6A}"/>
   </bookViews>
@@ -18,7 +18,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">ERC_SpD_spatial_registration_an!$A$1:$E$1</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="0" calcOnSave="0" concurrentCalc="0"/>
 </workbook>
 </file>
 
@@ -115,9 +115,6 @@
     <t>L2.3</t>
   </si>
   <si>
-    <t>L4.inhib</t>
-  </si>
-  <si>
     <t>L3</t>
   </si>
   <si>
@@ -134,6 +131,9 @@
   </si>
   <si>
     <t>Vasc</t>
+  </si>
+  <si>
+    <t>LD</t>
   </si>
 </sst>
 </file>
@@ -1015,7 +1015,7 @@
         <v>27</v>
       </c>
       <c r="E1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
@@ -1029,7 +1029,7 @@
         <v>23</v>
       </c>
       <c r="D2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E2">
         <v>1</v>
@@ -1046,7 +1046,7 @@
         <v>16</v>
       </c>
       <c r="D3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E3">
         <v>2</v>
@@ -1080,7 +1080,7 @@
         <v>5</v>
       </c>
       <c r="D5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E5">
         <v>4</v>
@@ -1097,7 +1097,7 @@
         <v>26</v>
       </c>
       <c r="D6" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="E6">
         <v>5</v>
@@ -1114,7 +1114,7 @@
         <v>10</v>
       </c>
       <c r="D7" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E7">
         <v>6</v>
@@ -1131,7 +1131,7 @@
         <v>13</v>
       </c>
       <c r="D8" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E8">
         <v>7</v>

</xml_diff>

<commit_message>
Update SpD annotation LD to Inhib
</commit_message>
<xml_diff>
--- a/processed-data/05_spe_correct_cluster/10_spatial_registration_DLPFC/ERC_SpD_spatial_registration_Annotations.xlsx
+++ b/processed-data/05_spe_correct_cluster/10_spatial_registration_DLPFC/ERC_SpD_spatial_registration_Annotations.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10420"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://lieberinstitute-my.sharepoint.com/personal/louise_huuki_libd_org/Documents/LIBD_code/LFF_spatial_ERC/processed-data/05_spe_correct_cluster/10_spatial_registration_DLPFC/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="31" documentId="8_{A6B8FFDE-9993-5E49-A3D7-A78A78ED7963}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{66F9A689-F83F-164C-8E66-69B4D30EDD03}"/>
+  <xr:revisionPtr revIDLastSave="32" documentId="8_{A6B8FFDE-9993-5E49-A3D7-A78A78ED7963}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CC8F0C2F-354E-9948-8A1D-8B018847C7A0}"/>
   <bookViews>
     <workbookView xWindow="1100" yWindow="820" windowWidth="28040" windowHeight="17440" xr2:uid="{145CA205-9E01-CF4B-AF13-75949B1F1E6A}"/>
   </bookViews>
@@ -18,7 +18,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">ERC_SpD_spatial_registration_an!$A$1:$E$1</definedName>
   </definedNames>
-  <calcPr calcId="0" calcOnSave="0" concurrentCalc="0"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
@@ -133,7 +133,7 @@
     <t>Vasc</t>
   </si>
   <si>
-    <t>LD</t>
+    <t>Inhib</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Update SpD annotation from L3 to LD
</commit_message>
<xml_diff>
--- a/processed-data/05_spe_correct_cluster/10_spatial_registration_DLPFC/ERC_SpD_spatial_registration_Annotations.xlsx
+++ b/processed-data/05_spe_correct_cluster/10_spatial_registration_DLPFC/ERC_SpD_spatial_registration_Annotations.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://lieberinstitute-my.sharepoint.com/personal/louise_huuki_libd_org/Documents/LIBD_code/LFF_spatial_ERC/processed-data/05_spe_correct_cluster/10_spatial_registration_DLPFC/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="32" documentId="8_{A6B8FFDE-9993-5E49-A3D7-A78A78ED7963}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CC8F0C2F-354E-9948-8A1D-8B018847C7A0}"/>
+  <xr:revisionPtr revIDLastSave="33" documentId="8_{A6B8FFDE-9993-5E49-A3D7-A78A78ED7963}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{398CA9CE-AFB2-504B-9F80-D4086A0A8F38}"/>
   <bookViews>
     <workbookView xWindow="1100" yWindow="820" windowWidth="28040" windowHeight="17440" xr2:uid="{145CA205-9E01-CF4B-AF13-75949B1F1E6A}"/>
   </bookViews>
@@ -115,9 +115,6 @@
     <t>L2.3</t>
   </si>
   <si>
-    <t>L3</t>
-  </si>
-  <si>
     <t>L5</t>
   </si>
   <si>
@@ -131,6 +128,9 @@
   </si>
   <si>
     <t>Vasc</t>
+  </si>
+  <si>
+    <t>LD</t>
   </si>
   <si>
     <t>Inhib</t>
@@ -1015,7 +1015,7 @@
         <v>27</v>
       </c>
       <c r="E1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
@@ -1029,7 +1029,7 @@
         <v>23</v>
       </c>
       <c r="D2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E2">
         <v>1</v>
@@ -1046,7 +1046,7 @@
         <v>16</v>
       </c>
       <c r="D3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E3">
         <v>2</v>
@@ -1080,7 +1080,7 @@
         <v>5</v>
       </c>
       <c r="D5" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="E5">
         <v>4</v>
@@ -1114,7 +1114,7 @@
         <v>10</v>
       </c>
       <c r="D7" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E7">
         <v>6</v>
@@ -1131,7 +1131,7 @@
         <v>13</v>
       </c>
       <c r="D8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E8">
         <v>7</v>

</xml_diff>